<commit_message>
adjust params for new term names.
</commit_message>
<xml_diff>
--- a/imgstat_props.xlsx
+++ b/imgstat_props.xlsx
@@ -46,19 +46,19 @@
     <t xml:space="preserve">trait_repeat_type</t>
   </si>
   <si>
-    <t xml:space="preserve">has_color_card</t>
+    <t xml:space="preserve">Color Card Present</t>
   </si>
   <si>
     <t xml:space="preserve">boolean</t>
   </si>
   <si>
-    <t xml:space="preserve">has_size_marker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">analysis_pass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_type</t>
+    <t xml:space="preserve">Size Marker Present</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analysis Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Type</t>
   </si>
   <si>
     <t xml:space="preserve">categorical</t>
@@ -67,52 +67,52 @@
     <t xml:space="preserve">fruit/seed/leaf/root/shoot</t>
   </si>
   <si>
-    <t xml:space="preserve">obj_count</t>
+    <t xml:space="preserve">Object Count</t>
   </si>
   <si>
     <t xml:space="preserve">numeric</t>
   </si>
   <si>
-    <t xml:space="preserve">obj_area_mask</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_area_hull</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_diam_max_ellipse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_diam_min_ellipse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_perimeter_mask</t>
+    <t xml:space="preserve">Object Area From Segmentation Mask</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Convex Hull Area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Maximum Diameter From Fitted Ellipse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Minimum Diameter From Fitted Ellipse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Perimeter From Segmentation Mask</t>
   </si>
   <si>
     <t xml:space="preserve">                                                                            </t>
   </si>
   <si>
-    <t xml:space="preserve">obj_solidity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_height</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_width</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_longest_path</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_aspect_ratio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_hull_vertices</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_ellipse_eccentricity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obj_ellipse_major_angle</t>
+    <t xml:space="preserve">Object Solidity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Height</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Width</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Longest Path</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Aspect Ratio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Convex Hull Vertices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Ellipse Eccentricity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object Ellipse Major Axis Angle</t>
   </si>
 </sst>
 </file>
@@ -122,11 +122,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -142,6 +143,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -186,9 +194,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -321,182 +337,182 @@
   <dimension ref="A1:H19"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.03"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>